<commit_message>
add multi-column merge selection
</commit_message>
<xml_diff>
--- a/sample_data/Testfile1.xlsx
+++ b/sample_data/Testfile1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\DataCombiner\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B13C535F-1C6F-4ECF-BC97-E21A172E4B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E53F54-C361-4824-A7BE-5AA7415167D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6915" yWindow="5205" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -382,7 +382,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>